<commit_message>
Prepare isolated production-synced iOS build with guarded manual CI
</commit_message>
<xml_diff>
--- a/public/ogrenci-veli-bilgi-formu.xlsx
+++ b/public/ogrenci-veli-bilgi-formu.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kayıtlar" sheetId="1" r:id="Rff3adcffeef343a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="Rbc3964e97ac3467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kayıtlar" sheetId="1" r:id="R4bdc9ea43ab34674"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Açıklamalar" sheetId="2" r:id="Re81a0d418a844a05"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -24,9 +24,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Veli Telefonu</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Her öğrenci için kendi satırındaki Sınıf/Şube bilgisini girin. Satırlar karışık sınıflarda olabilir. En fazla 500 kayıt ekleyin.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Telefon örnekleri: 05334138206, 5334138206, 905334138206 veya +905334138206.</x:t>
@@ -3835,8 +3832,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" t="s">
-        <x:v>5</x:v>
+      <x:c r="A1" t="str">
+        <x:v>Öğrenci sayısı kotası yoktur. Aktarım güvenli partiler halinde yapılır.</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -3846,12 +3843,12 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="s">
-        <x:v>6</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="s">
-        <x:v>7</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>